<commit_message>
feat(imm00): enhance bulk import, ref-data views, location simplify
- BE import: import_data.py +71 (endpoints), import_validators.py
  +257 (validation rules), import_helpers.py +194 (parse/folder/map)
- BE: ac_location.json — simplify contacts; patch v3_1/007 migrate
- FE list views: DeviceModelListView (+325), UserProfileListView (+302),
  ServiceContractListView (+318), SupplierListView (+341) — filter/CRUD
- FE: AssetCreateView, DeviceModelFormView, ReferenceDataView,
  types/import.ts — wire import wizard + form tweaks
- Assets: 9 Excel import templates refreshed
- Docs: imm-15/imm-16 sync, imports/generate_templates.py,
  res/plans/2026-05-19-drop-gmdn-status.md
- Chore: .claude settings + skills README, assetcore-commit skill
</commit_message>
<xml_diff>
--- a/assetcore/public/import_templates/01c_vi_tri.xlsx
+++ b/assetcore/public/import_templates/01c_vi_tri.xlsx
@@ -536,8 +536,8 @@
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -581,12 +581,12 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>emergency_contact</t>
+          <t>dept_head</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>dept_head</t>
+          <t>contact_phone</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -628,12 +628,12 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Liên hệ khẩn cấp</t>
+          <t>Người phụ trách (email)</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Trưởng khu vực (email)</t>
+          <t>Số liên hệ</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -675,12 +675,12 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Số DT hoặc email liên hệ khẩn cấp.</t>
+          <t>Email User phụ trách vị trí.</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Email User phụ trách vị trí.</t>
+          <t>Số liên hệ. Khi để trống, hệ thống sẽ tự lấy theo số di động của người phụ trách (mobile_no).</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -722,12 +722,12 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
+          <t>nguyen.van.a@hospital.vn</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
           <t>0901234567</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>nguyen.van.a@hospital.vn</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">

</xml_diff>